<commit_message>
Update reports 2026-10-23 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-10-23.xlsx
+++ b/gex_pivot_levels_2026-10-23.xlsx
@@ -15,12 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Pivots" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NQ'!$A$1:$G$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RTY'!$A$1:$G$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CL'!$A$1:$G$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GC'!$A$1:$G$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -602,12 +602,12 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>-$8.07M</t>
+          <t>-$9.68M</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>+$8.46M</t>
+          <t>+$10.16M</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -635,12 +635,12 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>-$1.76M</t>
+          <t>-$2.22M</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>+$2.30M</t>
+          <t>+$2.90M</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -685,266 +685,262 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
+        <v>7617.57</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>7580</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>-$7.02M</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>+$8.00M</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
         <v>7631.18</v>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B8" s="2" t="n">
         <v>757</v>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>-$13.45M</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>+$20.33M</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="n">
+      <c r="G8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
         <v>7637.57</v>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B9" s="5" t="n">
         <v>7600</v>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>-$20.48M</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>+$30.65M</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>-$24.09M</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>+$36.05M</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
+    <row r="10">
+      <c r="A10" s="2" t="n">
         <v>7642.57</v>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B10" s="2" t="n">
         <v>7605</v>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>-$1.63M</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>+$11.06M</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>-$1.89M</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>+$12.85M</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="n">
-        <v>7661.28</v>
-      </c>
-      <c r="B10" s="5" t="n">
-        <v>760</v>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>-$51.34M</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>+$63.60M</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
+        <v>7661.28</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>760</v>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>-$51.34M</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>+$63.60M</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
         <v>7662.57</v>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B12" s="5" t="n">
         <v>7625</v>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>-$11.64M</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>+$18.15M</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>-$13.06M</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>+$20.54M</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>7681.34</v>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>762</v>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>-$29.45M</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>+$40.84M</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
+        <v>7681.34</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>762</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>-$29.45M</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>+$40.84M</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
         <v>7682.57</v>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B14" s="2" t="n">
         <v>7645</v>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>-$4.25M</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>+$8.87M</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>-$4.62M</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>+$9.65M</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="n">
-        <v>7687.57</v>
-      </c>
-      <c r="B14" s="5" t="n">
-        <v>7650</v>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>-$19.59M</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>+$42.81M</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
-        <v>7697.57</v>
+        <v>7687.57</v>
       </c>
       <c r="B15" s="5" t="n">
-        <v>7660</v>
+        <v>7650</v>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
@@ -953,12 +949,12 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>-$656.60K</t>
+          <t>-$20.92M</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>+$19.74M</t>
+          <t>+$45.72M</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -968,96 +964,92 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
+        <v>7697.57</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>7660</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>-$677.45K</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>+$20.36M</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
         <v>7701.4</v>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B17" s="2" t="n">
         <v>764</v>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>-$13.27M</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>+$26.83M</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="n">
-        <v>7711.43</v>
-      </c>
-      <c r="B17" s="5" t="n">
-        <v>765</v>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>-$53.35M</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>+$82.23M</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
-        <v>7712.57</v>
+        <v>7711.43</v>
       </c>
       <c r="B18" s="5" t="n">
-        <v>7675</v>
+        <v>765</v>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>-$4.93M</t>
+          <t>-$53.35M</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>+$14.72M</t>
+          <t>+$82.23M</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -1073,241 +1065,237 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
+        <v>7712.57</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>7675</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>-$4.86M</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>+$14.50M</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
         <v>7721.46</v>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B20" s="2" t="n">
         <v>766</v>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>-$3.06M</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>+$24.74M</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="5" t="n">
+    <row r="21">
+      <c r="A21" s="5" t="n">
         <v>7731.49</v>
       </c>
-      <c r="B20" s="5" t="n">
+      <c r="B21" s="5" t="n">
         <v>767</v>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>-$30.36M</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>+$50.22M</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
+    <row r="22">
+      <c r="A22" s="2" t="n">
         <v>7732.57</v>
       </c>
-      <c r="B21" s="2" t="n">
+      <c r="B22" s="2" t="n">
         <v>7695</v>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>+$902.75K</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>+$10.06M</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>+$829.95K</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>+$9.25M</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="5" t="n">
+    <row r="23">
+      <c r="A23" s="5" t="n">
         <v>7737.57</v>
       </c>
-      <c r="B22" s="5" t="n">
+      <c r="B23" s="5" t="n">
         <v>7700</v>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>-$6.70M</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>+$53.68M</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>-$6.03M</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>+$48.31M</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
+    <row r="24">
+      <c r="A24" s="2" t="n">
         <v>7741.53</v>
       </c>
-      <c r="B23" s="2" t="n">
+      <c r="B24" s="2" t="n">
         <v>768</v>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>-$3.68M</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>+$38.28M</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="5" t="n">
+    <row r="25">
+      <c r="A25" s="5" t="n">
         <v>7751.56</v>
       </c>
-      <c r="B24" s="5" t="n">
+      <c r="B25" s="5" t="n">
         <v>769</v>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>-$84.32M</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>+$103.01M</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
-        <v>7757.57</v>
-      </c>
-      <c r="B25" s="2" t="n">
-        <v>7720</v>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>+$6.72M</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>+$15.32M</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>7762.57</v>
+        <v>7757.57</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>7725</v>
+        <v>7720</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
@@ -1316,27 +1304,31 @@
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>+$4.91M</t>
+          <t>+$5.46M</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>+$28.37M</t>
+          <t>+$12.45M</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>7777.57</v>
+        <v>7762.57</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>7740</v>
+        <v>7725</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
@@ -1345,12 +1337,12 @@
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>+$4.00M</t>
+          <t>+$3.91M</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>+$11.71M</t>
+          <t>+$22.57M</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -1362,35 +1354,64 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
+        <v>7777.57</v>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>7740</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>+$3.13M</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>+$9.15M</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
         <v>7787.57</v>
       </c>
-      <c r="B28" s="2" t="n">
+      <c r="B29" s="2" t="n">
         <v>7750</v>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>+$4.30M</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>+$26.00M</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>+$3.10M</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>+$18.72M</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr"/>
+      <c r="G29" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G28"/>
+  <autoFilter ref="A1:G29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3455,7 +3476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H85"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3707,24 +3728,24 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>7737.57</v>
+        <v>7731.49</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>7700</v>
+        <v>767</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>-$6.70M</t>
+          <t>-$30.36M</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>+$53.68M</t>
+          <t>+$50.22M</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -3745,24 +3766,24 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>7731.49</v>
+        <v>7737.57</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>767</v>
+        <v>7700</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>-$30.36M</t>
+          <t>-$6.03M</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>+$50.22M</t>
+          <t>+$48.31M</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -3795,12 +3816,12 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>-$19.59M</t>
+          <t>-$20.92M</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>+$42.81M</t>
+          <t>+$45.72M</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -3963,38 +3984,42 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>2816.8</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>280</v>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>+$26.32M</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>+$34.99M</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr"/>
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>7637.57</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>7600</v>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>-$24.09M</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>+$36.05M</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -4003,72 +4028,68 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
+        <v>2816.8</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>+$26.32M</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>+$34.99M</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
         <v>2826.86</v>
       </c>
-      <c r="C15" s="2" t="n">
+      <c r="C16" s="2" t="n">
         <v>281</v>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>+$28.02M</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>+$30.92M</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>7637.57</v>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>7600</v>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>-$20.48M</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>+$30.65M</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
@@ -4079,24 +4100,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>7762.57</v>
+        <v>7611.12</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>7725</v>
+        <v>755</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>+$4.91M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>-$17.60M</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>+$28.37M</t>
+          <t>+$27.83M</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -4113,10 +4134,10 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>7611.12</v>
+        <v>7701.4</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>755</v>
+        <v>764</v>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
@@ -4125,20 +4146,24 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>-$17.60M</t>
+          <t>-$13.27M</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>+$27.83M</t>
+          <t>+$26.83M</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -4147,10 +4172,10 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>7701.4</v>
+        <v>7721.46</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>764</v>
+        <v>766</v>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
@@ -4159,12 +4184,12 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>-$13.27M</t>
+          <t>-$3.06M</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>+$26.83M</t>
+          <t>+$24.74M</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -4181,28 +4206,28 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>7787.57</v>
+        <v>29598.86</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>7750</v>
+        <v>715</v>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>+$4.30M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>-$16.24M</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>+$26.00M</t>
+          <t>+$24.40M</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -4219,36 +4244,32 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>7721.46</v>
+        <v>7762.57</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>766</v>
+        <v>7725</v>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>-$3.06M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>+$3.91M</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>+$24.74M</t>
+          <t>+$22.57M</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -4257,10 +4278,10 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>29598.86</v>
+        <v>29804.39</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>715</v>
+        <v>720</v>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
@@ -4269,12 +4290,12 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>-$16.24M</t>
+          <t>-$10.18M</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>+$24.40M</t>
+          <t>+$22.02M</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -4287,72 +4308,76 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>29804.39</v>
+        <v>2756.44</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>720</v>
+        <v>274</v>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>-$10.18M</t>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>+$1.59M</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>+$22.02M</t>
+          <t>+$20.73M</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="n">
-        <v>2756.44</v>
-      </c>
-      <c r="C24" s="2" t="n">
-        <v>274</v>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>+$1.59M</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>+$20.73M</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>7662.57</v>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>7625</v>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>-$13.06M</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>+$20.54M</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -4363,70 +4388,66 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
+        <v>7697.57</v>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>7660</v>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>-$677.45K</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>+$20.36M</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
         <v>7631.18</v>
       </c>
-      <c r="C25" s="2" t="n">
+      <c r="C26" s="2" t="n">
         <v>757</v>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>-$13.45M</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>+$20.33M</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="n">
-        <v>7697.57</v>
-      </c>
-      <c r="C26" s="5" t="n">
-        <v>7660</v>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>-$656.60K</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>+$19.74M</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="H26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -4463,42 +4484,38 @@
       <c r="H27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B28" s="5" t="n">
-        <v>7662.57</v>
-      </c>
-      <c r="C28" s="5" t="n">
-        <v>7625</v>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="B28" s="2" t="n">
+        <v>7787.57</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>7750</v>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr">
-        <is>
-          <t>-$11.64M</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>+$18.15M</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>+$3.10M</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>+$18.72M</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -4507,36 +4524,32 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>7757.57</v>
+        <v>7510.81</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>7720</v>
+        <v>745</v>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E29" s="8" t="inlineStr">
-        <is>
-          <t>+$6.72M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>-$14.85M</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>+$15.32M</t>
+          <t>+$15.16M</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -4545,10 +4558,10 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>7510.81</v>
+        <v>7560.96</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>745</v>
+        <v>750</v>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
@@ -4557,12 +4570,12 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>-$14.85M</t>
+          <t>-$12.19M</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>+$15.16M</t>
+          <t>+$14.87M</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -4579,24 +4592,24 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>7560.96</v>
+        <v>7712.57</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>750</v>
+        <v>7675</v>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>-$12.19M</t>
+          <t>-$4.86M</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>+$14.87M</t>
+          <t>+$14.50M</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -4607,76 +4620,76 @@
       <c r="H31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="n">
-        <v>7712.57</v>
-      </c>
-      <c r="C32" s="5" t="n">
-        <v>7675</v>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="inlineStr">
-        <is>
-          <t>-$4.93M</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>+$14.72M</t>
-        </is>
-      </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H32" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>28571.18</v>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>690</v>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>-$13.98M</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>+$14.48M</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>28571.18</v>
+        <v>7642.57</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>690</v>
+        <v>7605</v>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>-$13.98M</t>
+          <t>-$1.89M</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>+$14.48M</t>
+          <t>+$12.85M</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -4685,10 +4698,10 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>7777.57</v>
+        <v>7757.57</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>7740</v>
+        <v>7720</v>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
@@ -4697,92 +4710,96 @@
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>+$4.00M</t>
+          <t>+$5.46M</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>+$11.71M</t>
+          <t>+$12.45M</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>2846.98</v>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>283</v>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>+$10.66M</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>+$10.66M</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B35" s="2" t="n">
-        <v>7642.57</v>
-      </c>
-      <c r="C35" s="2" t="n">
-        <v>7605</v>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="B36" s="5" t="n">
+        <v>7587.57</v>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>7550</v>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>-$1.63M</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>+$11.06M</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="n">
-        <v>2846.98</v>
-      </c>
-      <c r="C36" s="2" t="n">
-        <v>283</v>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>+$10.66M</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>+$10.66M</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="inlineStr"/>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>-$9.68M</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>+$10.16M</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -4791,24 +4808,24 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>7732.57</v>
+        <v>7682.57</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>7695</v>
+        <v>7645</v>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>+$902.75K</t>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>-$4.62M</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>+$10.06M</t>
+          <t>+$9.65M</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -4829,24 +4846,24 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>7682.57</v>
+        <v>7732.57</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>7645</v>
+        <v>7695</v>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>-$4.25M</t>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>+$829.95K</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>+$8.87M</t>
+          <t>+$9.25M</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -4861,42 +4878,38 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="inlineStr">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B39" s="5" t="n">
-        <v>7587.57</v>
-      </c>
-      <c r="C39" s="5" t="n">
-        <v>7550</v>
-      </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="B39" s="2" t="n">
+        <v>7777.57</v>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>7740</v>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E39" s="7" t="inlineStr">
-        <is>
-          <t>-$8.07M</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="inlineStr">
-        <is>
-          <t>+$8.46M</t>
-        </is>
-      </c>
-      <c r="G39" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H39" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>+$3.13M</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>+$9.15M</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
@@ -4975,42 +4988,38 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="n">
-        <v>3964.57</v>
-      </c>
-      <c r="C42" s="5" t="n">
-        <v>363</v>
-      </c>
-      <c r="D42" s="6" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr">
-        <is>
-          <t>-$6.74M</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="inlineStr">
-        <is>
-          <t>+$6.78M</t>
-        </is>
-      </c>
-      <c r="G42" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H42" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>7617.57</v>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>7580</v>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>-$7.02M</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>+$8.00M</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
@@ -5019,10 +5028,10 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>3986.41</v>
+        <v>3964.57</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
@@ -5031,12 +5040,12 @@
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>-$5.57M</t>
+          <t>-$6.74M</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>+$5.82M</t>
+          <t>+$6.78M</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
@@ -5057,110 +5066,110 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
+        <v>3986.41</v>
+      </c>
+      <c r="C44" s="5" t="n">
+        <v>365</v>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>-$5.57M</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>+$5.82M</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
         <v>3996.06</v>
       </c>
-      <c r="C44" s="5" t="n">
+      <c r="C45" s="5" t="n">
         <v>81</v>
       </c>
-      <c r="D44" s="6" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E44" s="7" t="inlineStr">
+      <c r="E45" s="7" t="inlineStr">
         <is>
           <t>-$5.11M</t>
         </is>
       </c>
-      <c r="F44" s="6" t="inlineStr">
+      <c r="F45" s="6" t="inlineStr">
         <is>
           <t>+$5.12M</t>
         </is>
       </c>
-      <c r="G44" s="6" t="inlineStr">
+      <c r="G45" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H44" s="6" t="inlineStr">
+      <c r="H45" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B45" s="2" t="n">
+      <c r="B46" s="2" t="n">
         <v>29311.11</v>
       </c>
-      <c r="C45" s="2" t="n">
+      <c r="C46" s="2" t="n">
         <v>708</v>
       </c>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="D46" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="E46" s="4" t="inlineStr">
         <is>
           <t>-$2.62M</t>
         </is>
       </c>
-      <c r="F45" s="3" t="inlineStr">
+      <c r="F46" s="3" t="inlineStr">
         <is>
           <t>+$4.78M</t>
         </is>
       </c>
-      <c r="G45" s="3" t="inlineStr">
+      <c r="G46" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr">
+      <c r="H46" s="3" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="n">
-        <v>3931.8</v>
-      </c>
-      <c r="C46" s="5" t="n">
-        <v>360</v>
-      </c>
-      <c r="D46" s="6" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E46" s="7" t="inlineStr">
-        <is>
-          <t>-$4.54M</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="inlineStr">
-        <is>
-          <t>+$4.75M</t>
-        </is>
-      </c>
-      <c r="G46" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H46" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
@@ -5171,10 +5180,10 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>4062.87</v>
+        <v>3931.8</v>
       </c>
       <c r="C47" s="5" t="n">
-        <v>372</v>
+        <v>360</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
@@ -5183,12 +5192,12 @@
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>-$4.39M</t>
+          <t>-$4.54M</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>+$4.52M</t>
+          <t>+$4.75M</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">
@@ -5205,28 +5214,28 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>98.45</v>
+        <v>4062.87</v>
       </c>
       <c r="C48" s="5" t="n">
-        <v>160</v>
+        <v>372</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E48" s="9" t="inlineStr">
-        <is>
-          <t>+$2.10M</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>-$4.39M</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>+$3.93M</t>
+          <t>+$4.52M</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr">
@@ -5236,35 +5245,35 @@
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>4094.73</v>
+        <v>98.45</v>
       </c>
       <c r="C49" s="5" t="n">
-        <v>83</v>
+        <v>160</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E49" s="7" t="inlineStr">
-        <is>
-          <t>-$2.65M</t>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>+$2.10M</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr">
         <is>
-          <t>+$3.29M</t>
+          <t>+$3.93M</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr">
@@ -5274,7 +5283,7 @@
       </c>
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -5285,70 +5294,74 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
+        <v>4094.73</v>
+      </c>
+      <c r="C50" s="5" t="n">
+        <v>83</v>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>-$2.65M</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>+$3.29M</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
         <v>4193.4</v>
       </c>
-      <c r="C50" s="5" t="n">
+      <c r="C51" s="5" t="n">
         <v>85</v>
       </c>
-      <c r="D50" s="6" t="inlineStr">
+      <c r="D51" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E50" s="7" t="inlineStr">
+      <c r="E51" s="7" t="inlineStr">
         <is>
           <t>-$2.86M</t>
         </is>
       </c>
-      <c r="F50" s="6" t="inlineStr">
+      <c r="F51" s="6" t="inlineStr">
         <is>
           <t>+$3.04M</t>
         </is>
       </c>
-      <c r="G50" s="6" t="inlineStr">
+      <c r="G51" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H50" s="6" t="inlineStr">
+      <c r="H51" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="n">
-        <v>4095.63</v>
-      </c>
-      <c r="C51" s="2" t="n">
-        <v>375</v>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t>-$380.20K</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
-          <t>+$2.88M</t>
-        </is>
-      </c>
-      <c r="G51" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -5369,12 +5382,12 @@
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>-$1.76M</t>
+          <t>-$2.22M</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>+$2.30M</t>
+          <t>+$2.90M</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
@@ -5395,36 +5408,32 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>4144.06</v>
+        <v>4095.63</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>84</v>
+        <v>375</v>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>-$453.82K</t>
+          <t>-$380.20K</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>+$1.65M</t>
+          <t>+$2.88M</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H53" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
@@ -5433,24 +5442,24 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>4019.18</v>
+        <v>4144.06</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>368</v>
+        <v>84</v>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>-$1.07M</t>
+          <t>-$453.82K</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>+$1.46M</t>
+          <t>+$1.65M</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
@@ -5471,168 +5480,168 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>4150.24</v>
+        <v>4019.18</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>380</v>
+        <v>368</v>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>+$811.76K</t>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>-$1.07M</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>+$1.45M</t>
+          <t>+$1.46M</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H55" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="n">
+        <v>4150.24</v>
+      </c>
+      <c r="C56" s="2" t="n">
+        <v>380</v>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>+$811.76K</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>+$1.45M</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B56" s="2" t="n">
+      <c r="B57" s="2" t="n">
         <v>104.6</v>
       </c>
-      <c r="C56" s="2" t="n">
+      <c r="C57" s="2" t="n">
         <v>170</v>
       </c>
-      <c r="D56" s="3" t="inlineStr">
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E56" s="8" t="inlineStr">
+      <c r="E57" s="8" t="inlineStr">
         <is>
           <t>+$1.39M</t>
         </is>
       </c>
-      <c r="F56" s="3" t="inlineStr">
+      <c r="F57" s="3" t="inlineStr">
         <is>
           <t>+$1.43M</t>
         </is>
       </c>
-      <c r="G56" s="3" t="inlineStr">
+      <c r="G57" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H56" s="3" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="6" t="inlineStr">
+      <c r="H57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B57" s="5" t="n">
+      <c r="B58" s="5" t="n">
         <v>3848.06</v>
       </c>
-      <c r="C57" s="5" t="n">
+      <c r="C58" s="5" t="n">
         <v>78</v>
       </c>
-      <c r="D57" s="6" t="inlineStr">
+      <c r="D58" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E57" s="7" t="inlineStr">
+      <c r="E58" s="7" t="inlineStr">
         <is>
           <t>-$1.42M</t>
         </is>
       </c>
-      <c r="F57" s="6" t="inlineStr">
+      <c r="F58" s="6" t="inlineStr">
         <is>
           <t>+$1.43M</t>
         </is>
       </c>
-      <c r="G57" s="6" t="inlineStr">
+      <c r="G58" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H57" s="6" t="inlineStr">
+      <c r="H58" s="6" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="n">
-        <v>4051.94</v>
-      </c>
-      <c r="C58" s="2" t="n">
-        <v>371</v>
-      </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E58" s="4" t="inlineStr">
-        <is>
-          <t>-$1.11M</t>
-        </is>
-      </c>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
-          <t>+$1.38M</t>
-        </is>
-      </c>
-      <c r="G58" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H58" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>99.06</v>
+        <v>4051.94</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>161</v>
+        <v>371</v>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E59" s="8" t="inlineStr">
-        <is>
-          <t>+$524.61K</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>-$1.11M</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>+$1.34M</t>
+          <t>+$1.38M</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
@@ -5642,7 +5651,7 @@
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -5653,104 +5662,108 @@
         </is>
       </c>
       <c r="B60" s="2" t="n">
+        <v>99.06</v>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>161</v>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>+$524.61K</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>+$1.34M</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="n">
         <v>96.59999999999999</v>
       </c>
-      <c r="C60" s="2" t="n">
+      <c r="C61" s="2" t="n">
         <v>157</v>
       </c>
-      <c r="D60" s="3" t="inlineStr">
+      <c r="D61" s="3" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E60" s="8" t="inlineStr">
+      <c r="E61" s="8" t="inlineStr">
         <is>
           <t>+$566.59K</t>
         </is>
       </c>
-      <c r="F60" s="3" t="inlineStr">
+      <c r="F61" s="3" t="inlineStr">
         <is>
           <t>+$1.21M</t>
         </is>
       </c>
-      <c r="G60" s="3" t="inlineStr">
+      <c r="G61" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H60" s="3" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="6" t="inlineStr">
+      <c r="H61" s="3" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B61" s="5" t="n">
+      <c r="B62" s="5" t="n">
         <v>4341.4</v>
       </c>
-      <c r="C61" s="5" t="n">
+      <c r="C62" s="5" t="n">
         <v>88</v>
       </c>
-      <c r="D61" s="6" t="inlineStr">
+      <c r="D62" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E61" s="9" t="inlineStr">
+      <c r="E62" s="9" t="inlineStr">
         <is>
           <t>+$1.10M</t>
         </is>
       </c>
-      <c r="F61" s="6" t="inlineStr">
+      <c r="F62" s="6" t="inlineStr">
         <is>
           <t>+$1.17M</t>
         </is>
       </c>
-      <c r="G61" s="6" t="inlineStr">
+      <c r="G62" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H61" s="6" t="inlineStr">
+      <c r="H62" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="n">
-        <v>4390.73</v>
-      </c>
-      <c r="C62" s="2" t="n">
-        <v>89</v>
-      </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E62" s="8" t="inlineStr">
-        <is>
-          <t>+$872.73K</t>
-        </is>
-      </c>
-      <c r="F62" s="3" t="inlineStr">
-        <is>
-          <t>+$910.19K</t>
-        </is>
-      </c>
-      <c r="G62" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -5759,10 +5772,10 @@
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>4440.07</v>
+        <v>4390.73</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
@@ -5771,12 +5784,12 @@
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t>+$773.49K</t>
+          <t>+$872.73K</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>+$879.56K</t>
+          <t>+$910.19K</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
@@ -5793,24 +5806,24 @@
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>4204.85</v>
+        <v>4440.07</v>
       </c>
       <c r="C64" s="2" t="n">
-        <v>385</v>
+        <v>90</v>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
         <is>
-          <t>+$665.87K</t>
+          <t>+$773.49K</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>+$823.12K</t>
+          <t>+$879.56K</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
@@ -5827,104 +5840,104 @@
         </is>
       </c>
       <c r="B65" s="2" t="n">
+        <v>4204.85</v>
+      </c>
+      <c r="C65" s="2" t="n">
+        <v>385</v>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>+$665.87K</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>+$823.12K</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="n">
         <v>4588.07</v>
       </c>
-      <c r="C65" s="2" t="n">
+      <c r="C66" s="2" t="n">
         <v>93</v>
       </c>
-      <c r="D65" s="3" t="inlineStr">
+      <c r="D66" s="3" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E65" s="8" t="inlineStr">
+      <c r="E66" s="8" t="inlineStr">
         <is>
           <t>+$662.00K</t>
         </is>
       </c>
-      <c r="F65" s="3" t="inlineStr">
+      <c r="F66" s="3" t="inlineStr">
         <is>
           <t>+$686.79K</t>
         </is>
       </c>
-      <c r="G65" s="3" t="inlineStr">
+      <c r="G66" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H65" s="3" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="6" t="inlineStr">
+      <c r="H66" s="3" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B66" s="5" t="n">
+      <c r="B67" s="5" t="n">
         <v>29307.31</v>
       </c>
-      <c r="C66" s="5" t="n">
+      <c r="C67" s="5" t="n">
         <v>29100</v>
       </c>
-      <c r="D66" s="6" t="inlineStr">
+      <c r="D67" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E66" s="7" t="inlineStr">
+      <c r="E67" s="7" t="inlineStr">
         <is>
           <t>-$419.32K</t>
         </is>
       </c>
-      <c r="F66" s="6" t="inlineStr">
+      <c r="F67" s="6" t="inlineStr">
         <is>
           <t>+$683.43K</t>
         </is>
       </c>
-      <c r="G66" s="6" t="inlineStr">
+      <c r="G67" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H66" s="6" t="inlineStr">
+      <c r="H67" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="n">
-        <v>3700.06</v>
-      </c>
-      <c r="C67" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="D67" s="3" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E67" s="4" t="inlineStr">
-        <is>
-          <t>-$582.72K</t>
-        </is>
-      </c>
-      <c r="F67" s="3" t="inlineStr">
-        <is>
-          <t>+$585.71K</t>
-        </is>
-      </c>
-      <c r="G67" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
@@ -5933,24 +5946,24 @@
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>4538.73</v>
+        <v>3700.06</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E68" s="8" t="inlineStr">
-        <is>
-          <t>+$513.91K</t>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>-$582.72K</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>+$529.69K</t>
+          <t>+$585.71K</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
@@ -5967,36 +5980,32 @@
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>3975.49</v>
+        <v>4538.73</v>
       </c>
       <c r="C69" s="2" t="n">
-        <v>364</v>
+        <v>92</v>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>-$431.60K</t>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>+$513.91K</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>+$487.18K</t>
+          <t>+$529.69K</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H69" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
@@ -6005,184 +6014,184 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
+        <v>3975.49</v>
+      </c>
+      <c r="C70" s="2" t="n">
+        <v>364</v>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>-$431.60K</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>+$487.18K</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="n">
         <v>4070.06</v>
       </c>
-      <c r="C70" s="2" t="n">
+      <c r="C71" s="2" t="n">
         <v>82.5</v>
       </c>
-      <c r="D70" s="3" t="inlineStr">
+      <c r="D71" s="3" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E70" s="4" t="inlineStr">
+      <c r="E71" s="4" t="inlineStr">
         <is>
           <t>-$358.82K</t>
         </is>
       </c>
-      <c r="F70" s="3" t="inlineStr">
+      <c r="F71" s="3" t="inlineStr">
         <is>
           <t>+$378.29K</t>
         </is>
       </c>
-      <c r="G70" s="3" t="inlineStr">
+      <c r="G71" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H70" s="3" t="inlineStr">
+      <c r="H71" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="6" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B71" s="5" t="n">
+      <c r="B72" s="5" t="n">
         <v>29157.31</v>
       </c>
-      <c r="C71" s="5" t="n">
+      <c r="C72" s="5" t="n">
         <v>28950</v>
       </c>
-      <c r="D71" s="6" t="inlineStr">
+      <c r="D72" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E71" s="7" t="inlineStr">
+      <c r="E72" s="7" t="inlineStr">
         <is>
           <t>-$108.88K</t>
         </is>
       </c>
-      <c r="F71" s="6" t="inlineStr">
+      <c r="F72" s="6" t="inlineStr">
         <is>
           <t>+$192.29K</t>
         </is>
       </c>
-      <c r="G71" s="6" t="inlineStr">
+      <c r="G72" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H71" s="6" t="inlineStr">
+      <c r="H72" s="6" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="n">
-        <v>3942.73</v>
-      </c>
-      <c r="C72" s="2" t="n">
-        <v>361</v>
-      </c>
-      <c r="D72" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E72" s="4" t="inlineStr">
-        <is>
-          <t>-$167.85K</t>
-        </is>
-      </c>
-      <c r="F72" s="3" t="inlineStr">
-        <is>
-          <t>+$177.93K</t>
-        </is>
-      </c>
-      <c r="G72" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H72" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="n">
+        <v>3942.73</v>
+      </c>
+      <c r="C73" s="2" t="n">
+        <v>361</v>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>-$167.85K</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>+$177.93K</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B73" s="2" t="n">
+      <c r="B74" s="2" t="n">
         <v>29207.31</v>
       </c>
-      <c r="C73" s="2" t="n">
+      <c r="C74" s="2" t="n">
         <v>29000</v>
       </c>
-      <c r="D73" s="3" t="inlineStr">
+      <c r="D74" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E73" s="4" t="inlineStr">
+      <c r="E74" s="4" t="inlineStr">
         <is>
           <t>-$44.02K</t>
         </is>
       </c>
-      <c r="F73" s="3" t="inlineStr">
+      <c r="F74" s="3" t="inlineStr">
         <is>
           <t>+$150.59K</t>
         </is>
       </c>
-      <c r="G73" s="3" t="inlineStr">
+      <c r="G74" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H73" s="3" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B74" s="5" t="n">
-        <v>29107.31</v>
-      </c>
-      <c r="C74" s="5" t="n">
-        <v>28900</v>
-      </c>
-      <c r="D74" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E74" s="7" t="inlineStr">
-        <is>
-          <t>-$127.42K</t>
-        </is>
-      </c>
-      <c r="F74" s="6" t="inlineStr">
-        <is>
-          <t>+$150.59K</t>
-        </is>
-      </c>
-      <c r="G74" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H74" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
@@ -6191,72 +6200,72 @@
         </is>
       </c>
       <c r="B75" s="5" t="n">
+        <v>29107.31</v>
+      </c>
+      <c r="C75" s="5" t="n">
+        <v>28900</v>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>-$127.42K</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>+$150.59K</t>
+        </is>
+      </c>
+      <c r="G75" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="n">
         <v>29237.31</v>
       </c>
-      <c r="C75" s="5" t="n">
+      <c r="C76" s="5" t="n">
         <v>29030</v>
       </c>
-      <c r="D75" s="6" t="inlineStr">
+      <c r="D76" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E75" s="9" t="inlineStr">
+      <c r="E76" s="9" t="inlineStr">
         <is>
           <t>+$53.28K</t>
         </is>
       </c>
-      <c r="F75" s="6" t="inlineStr">
+      <c r="F76" s="6" t="inlineStr">
         <is>
           <t>+$118.15K</t>
         </is>
       </c>
-      <c r="G75" s="6" t="inlineStr">
+      <c r="G76" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H75" s="6" t="inlineStr">
+      <c r="H76" s="6" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B76" s="2" t="n">
-        <v>29177.31</v>
-      </c>
-      <c r="C76" s="2" t="n">
-        <v>28970</v>
-      </c>
-      <c r="D76" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E76" s="4" t="inlineStr">
-        <is>
-          <t>-$94.98K</t>
-        </is>
-      </c>
-      <c r="F76" s="3" t="inlineStr">
-        <is>
-          <t>+$108.88K</t>
-        </is>
-      </c>
-      <c r="G76" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H76" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
@@ -6267,10 +6276,10 @@
         </is>
       </c>
       <c r="B77" s="2" t="n">
-        <v>29127.31</v>
+        <v>29177.31</v>
       </c>
       <c r="C77" s="2" t="n">
-        <v>28920</v>
+        <v>28970</v>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
@@ -6279,20 +6288,24 @@
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>-$76.45K</t>
+          <t>-$94.98K</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>+$99.62K</t>
+          <t>+$108.88K</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H77" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
@@ -6301,106 +6314,102 @@
         </is>
       </c>
       <c r="B78" s="2" t="n">
+        <v>29127.31</v>
+      </c>
+      <c r="C78" s="2" t="n">
+        <v>28920</v>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>-$76.45K</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>+$99.62K</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="n">
         <v>29357.31</v>
       </c>
-      <c r="C78" s="2" t="n">
+      <c r="C79" s="2" t="n">
         <v>29150</v>
       </c>
-      <c r="D78" s="3" t="inlineStr">
+      <c r="D79" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E78" s="4" t="inlineStr">
+      <c r="E79" s="4" t="inlineStr">
         <is>
           <t>-$30.12K</t>
         </is>
       </c>
-      <c r="F78" s="3" t="inlineStr">
+      <c r="F79" s="3" t="inlineStr">
         <is>
           <t>+$99.62K</t>
         </is>
       </c>
-      <c r="G78" s="3" t="inlineStr">
+      <c r="G79" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H78" s="3" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="6" t="inlineStr">
+      <c r="H79" s="3" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B79" s="5" t="n">
+      <c r="B80" s="5" t="n">
         <v>29007.31</v>
       </c>
-      <c r="C79" s="5" t="n">
+      <c r="C80" s="5" t="n">
         <v>28800</v>
       </c>
-      <c r="D79" s="6" t="inlineStr">
+      <c r="D80" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E79" s="7" t="inlineStr">
+      <c r="E80" s="7" t="inlineStr">
         <is>
           <t>-$91.22K</t>
         </is>
       </c>
-      <c r="F79" s="6" t="inlineStr">
+      <c r="F80" s="6" t="inlineStr">
         <is>
           <t>+$99.33K</t>
         </is>
       </c>
-      <c r="G79" s="6" t="inlineStr">
+      <c r="G80" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H79" s="6" t="inlineStr">
+      <c r="H80" s="6" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B80" s="2" t="n">
-        <v>29267.31</v>
-      </c>
-      <c r="C80" s="2" t="n">
-        <v>29060</v>
-      </c>
-      <c r="D80" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E80" s="8" t="inlineStr">
-        <is>
-          <t>+$62.55K</t>
-        </is>
-      </c>
-      <c r="F80" s="3" t="inlineStr">
-        <is>
-          <t>+$81.08K</t>
-        </is>
-      </c>
-      <c r="G80" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H80" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
@@ -6411,24 +6420,24 @@
         </is>
       </c>
       <c r="B81" s="2" t="n">
-        <v>29167.31</v>
+        <v>29267.31</v>
       </c>
       <c r="C81" s="2" t="n">
-        <v>28960</v>
+        <v>29060</v>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E81" s="4" t="inlineStr">
-        <is>
-          <t>-$6.95K</t>
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t>+$62.55K</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>+$76.45K</t>
+          <t>+$81.08K</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -6445,28 +6454,28 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
-        <v>3897.39</v>
+        <v>29167.31</v>
       </c>
       <c r="C82" s="2" t="n">
-        <v>79</v>
+        <v>28960</v>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>NDX</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>-$46.74K</t>
+          <t>-$6.95K</t>
         </is>
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>+$74.65K</t>
+          <t>+$76.45K</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">
@@ -6483,28 +6492,28 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B83" s="2" t="n">
-        <v>29257.31</v>
+        <v>3897.39</v>
       </c>
       <c r="C83" s="2" t="n">
-        <v>29050</v>
+        <v>79</v>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>-$30.12K</t>
+          <t>-$46.74K</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>+$67.18K</t>
+          <t>+$74.65K</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
@@ -6514,7 +6523,7 @@
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -6525,10 +6534,10 @@
         </is>
       </c>
       <c r="B84" s="2" t="n">
-        <v>29032.31</v>
+        <v>29257.31</v>
       </c>
       <c r="C84" s="2" t="n">
-        <v>28825</v>
+        <v>29050</v>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
@@ -6537,12 +6546,12 @@
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>-$6.08K</t>
+          <t>-$30.12K</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>+$26.35K</t>
+          <t>+$67.18K</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
@@ -6552,7 +6561,7 @@
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -6563,39 +6572,77 @@
         </is>
       </c>
       <c r="B85" s="2" t="n">
+        <v>29032.31</v>
+      </c>
+      <c r="C85" s="2" t="n">
+        <v>28825</v>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>-$6.08K</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>+$26.35K</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="n">
         <v>29117.31</v>
       </c>
-      <c r="C85" s="2" t="n">
+      <c r="C86" s="2" t="n">
         <v>28910</v>
       </c>
-      <c r="D85" s="3" t="inlineStr">
+      <c r="D86" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E85" s="4" t="inlineStr">
+      <c r="E86" s="4" t="inlineStr">
         <is>
           <t>-$6.95K</t>
         </is>
       </c>
-      <c r="F85" s="3" t="inlineStr">
+      <c r="F86" s="3" t="inlineStr">
         <is>
           <t>+$6.95K</t>
         </is>
       </c>
-      <c r="G85" s="3" t="inlineStr">
+      <c r="G86" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H85" s="3" t="inlineStr">
+      <c r="H86" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H85"/>
+  <autoFilter ref="A1:H86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>